<commit_message>
update tables and plots output
</commit_message>
<xml_diff>
--- a/OMOP Analysis/Results/Table1_OMOP.xlsx
+++ b/OMOP Analysis/Results/Table1_OMOP.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -625,24 +625,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>No Visits</t>
+          <t>Visits with Non-clinically Relevant Staff</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>101 (13%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Visits with Non-clinically Relevant Staff</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>699 (87%)</t>
+          <t>800 (100%)</t>
         </is>
       </c>
     </row>

</xml_diff>